<commit_message>
fix: preserve character stature across story playback and editing
</commit_message>
<xml_diff>
--- a/docs/architecture/evidence/authoring-format/knolstory-blank-v2.xlsx
+++ b/docs/architecture/evidence/authoring-format/knolstory-blank-v2.xlsx
@@ -13003,7 +13003,7 @@
     <t>놀스토리</t>
   </si>
   <si>
-    <t>2026-10-28T23:25:20.766Z</t>
+    <t>2026-10-30T07:24:08.914Z</t>
   </si>
   <si>
     <t>knolstory-next</t>
@@ -13075,7 +13075,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-10-28T23:25:20.765Z</t>
+    <t>2026-10-30T07:24:08.913Z</t>
   </si>
   <si>
     <t>없음</t>

</xml_diff>